<commit_message>
nsamples + sensitivity analyses
</commit_message>
<xml_diff>
--- a/data/sensitivity_analyses.xlsx
+++ b/data/sensitivity_analyses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://burnetinstitute.sharepoint.com/sites/WG-Modelling-HCVvaccinemodel/Shared Documents/HCV vaccine model/HCV vaccine model/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\farah.houdroge\Documents\GitHub\hcv-vaccine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="233" documentId="8_{0F44D86B-B6ED-4572-A374-5733EC519498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA91EE4F-AE73-442B-B6B1-B359339AD983}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B9C321-14D6-420E-A026-B10070219F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1BA74FC1-72AA-40E0-9CB9-1F13813B1A51}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1BA74FC1-72AA-40E0-9CB9-1F13813B1A51}"/>
   </bookViews>
   <sheets>
     <sheet name="econ" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="84">
   <si>
     <t>scenario_name</t>
   </si>
@@ -324,6 +324,30 @@
   </si>
   <si>
     <t>G1 (%),G3 (%),G4 (%)</t>
+  </si>
+  <si>
+    <t>vax_cost_0</t>
+  </si>
+  <si>
+    <t>Vaccine unit cost $0</t>
+  </si>
+  <si>
+    <t>daa_cost_lower</t>
+  </si>
+  <si>
+    <t>DAA Treatment Lower</t>
+  </si>
+  <si>
+    <t>productivity_50</t>
+  </si>
+  <si>
+    <t>productivity_0</t>
+  </si>
+  <si>
+    <t>PWID employment 50%</t>
+  </si>
+  <si>
+    <t>PWID employment 0%</t>
   </si>
 </sst>
 </file>
@@ -733,13 +757,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED89CEC-CC02-4EE3-88DB-D6D932004621}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -747,7 +772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -755,7 +780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -763,7 +788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -771,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -779,7 +804,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -787,7 +812,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -795,7 +820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -803,12 +828,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>30</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -820,15 +877,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C4335FB-68B3-4701-A71F-5E327C9ABFD5}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7265625" customWidth="1"/>
     <col min="2" max="2" width="33" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -842,7 +899,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -856,7 +913,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -870,7 +927,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -884,7 +941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -898,7 +955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -912,7 +969,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -926,7 +983,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -940,7 +997,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -954,7 +1011,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -976,16 +1033,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E737958-3D4A-47AC-9212-F56E9F891CFE}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1059,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1019,7 +1076,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1036,7 +1093,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1053,7 +1110,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1070,7 +1127,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -1087,7 +1144,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1104,7 +1161,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1121,7 +1178,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1138,7 +1195,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1155,7 +1212,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1352,6 +1409,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="460e4ad2-c64b-4f67-8552-094351f252e3">
@@ -1359,15 +1425,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1389,6 +1446,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66F33292-D62A-45EC-AF26-63D12627EE36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED2B22C5-9244-4522-A6F2-56936D2B0CD3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1402,12 +1467,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66F33292-D62A-45EC-AF26-63D12627EE36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>